<commit_message>
fix: BEFR labels, remove branding from SOV, show keyword count, fix None sorting
</commit_message>
<xml_diff>
--- a/Keyword_Research_DeDecker_BENL_FINAL .xlsx
+++ b/Keyword_Research_DeDecker_BENL_FINAL .xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marc/Desktop/semantic_analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90411D0A-41B4-2444-852A-BAF6EAF93A45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B99D4DF4-5294-DD48-BD6D-F0B4E0C29416}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>